<commit_message>
Rework the literature spreadsheet: energy harvesting papers only, shorter descriptions, add a terms sheet
</commit_message>
<xml_diff>
--- a/docs/research/2026-09-20-energy-prediction-literature.xlsx
+++ b/docs/research/2026-09-20-energy-prediction-literature.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What we found" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Background" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What we found" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terms" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Papers'!$A$1:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Papers'!$A$1:$K$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,12 +54,18 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="00555555"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF1F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,7 +115,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,17 +486,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Energy prediction for our harvesting sensor nodes: literature review</t>
+          <t>Predicting harvested energy on solar sensor nodes: literature review</t>
         </is>
       </c>
     </row>
@@ -490,43 +508,43 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>20 September 2026, for the senior design project (sdp-sensor-nodes).</t>
+          <t>September 2026, for the senior design project (sdp-sensor-nodes).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Question behind it</t>
+          <t>The question</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>We want the VPS to predict how much energy each node will have, so it can decide which node gets the next task. Before building that, we wanted to know whether the field uses statistical methods or machine learning, and which one we should pick.</t>
+          <t>Our server should decide which node gets the next task, based on how much energy that node will have. Do we predict that with a statistical method or with machine learning?</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>What is in here</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>The Papers sheet summarises 14 studies. What we found records the conclusions we drew across them, including our own hardware numbers. Decision states what we plan to do and what would change our minds.</t>
+          <t>24 papers, all on energy harvesting nodes, solar prediction for those nodes, or scheduling tasks on them. Two general forecasting papers sit on the Background sheet because they are about retail and business data, not energy.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>How the papers were found</t>
+          <t>How to read the Papers sheet</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Searches across IEEE Xplore, the ACM Digital Library, arXiv, MDPI, Semantic Scholar and publisher pages, using AI research assistance. Every DOI and arXiv identifier was then checked against its Crossref or arXiv record for title, authors, venue and year.</t>
+          <t>Group says why the paper is here. What they did is the method in plain words. Setup says hardware or simulation and at what scale. Main result gives the numbers the paper reports. Why it matters says what we take from it.</t>
         </is>
       </c>
     </row>
@@ -538,7 +556,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Full text means we read the paper itself. Abstract only means we read the abstract or the publisher record, and nothing more. Preprint means it has not been peer reviewed.</t>
+          <t>Full text means we read the paper. Abstract only means we read the abstract or publisher record and nothing more. Preprint means not peer reviewed.</t>
         </is>
       </c>
     </row>
@@ -550,19 +568,19 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>An empty cell means we could not confirm that item from what we read. We did not fill gaps with guesses.</t>
+          <t>An empty cell means we could not confirm that item from what we read. Nothing is filled in by guesswork.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Numbers</t>
+          <t>Comparing numbers</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Figures are quoted as each paper reports them. Metrics, sites and horizons differ between papers, so compare within a paper rather than across them.</t>
+          <t>Metrics, sites and horizons differ between papers. Compare figures within a paper, not across papers.</t>
         </is>
       </c>
     </row>
@@ -574,19 +592,31 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Rows marked as ours in What we found come from our hardware and datasheets, not from the papers. They are calculations, and the PPK2 measurements will replace them.</t>
+          <t>Rows marked as ours on the What we found sheet come from our hardware and datasheets. They are calculations, and PPK2 measurements will replace them.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Checking</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Every DOI and arXiv identifier was checked against its Crossref or arXiv record for title, authors, venue and year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>AI disclosure</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>The search, extraction and drafting used AI assistance (Claude). Check any figure against the original before quoting it in the report.</t>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Searching, extraction and drafting used AI assistance (Claude). Verify any figure against the original before quoting it.</t>
         </is>
       </c>
     </row>
@@ -601,19 +631,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
-    <col width="56" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -624,47 +655,52 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Paper title</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Authors and year</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>Authors, year</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
           <t>Published in</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>What they covered</t>
-        </is>
-      </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Numbers they report</t>
+          <t>What they did</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>What they concluded</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>What it means for our project</t>
+          <t>Main result</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
+          <t>Why it matters to us</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>DOI or link</t>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
@@ -672,49 +708,50 @@
       <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Prediction and management in energy harvested wireless sensor nodes</t>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>A. Predicting harvest</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Recas Piorno, Bergonzini, Atienza and Simunic Rosing, 2009</t>
+          <t>Power management in energy harvesting sensor networks</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Wireless VITAE 2009, pages 6 to 10</t>
+          <t>Kansal, Hsu, Zahedi and Srivastava, 2007</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Introduces WCMA, a weather conditioned moving average. It predicts the next 30 minute slot of solar harvest from the last sample and the mean of the same slot over the previous four days, scaled by how today is running compared with those days. Tuned and tested on 45 days of one minute measurements from a PowerFilm panel on a supercapacitor node.</t>
+          <t>ACM TECS 6(4)</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Average prediction error 9.8 percent for WCMA against 28.6 percent for EWMA. On a day with a sudden weather change, the noon slot error was 10.20 percent for WCMA and minus 90.99 percent for EWMA.</t>
+          <t>Keeps a running average of how much each half hour of the day has harvested on past days, and sets the node's duty cycle from it, correcting as the day goes.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>A small amount of recent history, weighted by how the current day is running, predicts the next slot far better than an exponentially weighted average, at negligible cost on the node.</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>This is the cheap baseline any model on our server has to beat. The parameters were tuned on the same 45 days they were tested on, so read 9.8 percent as optimistic.</t>
-        </is>
-      </c>
+          <t>Method paper. No prediction error reported.</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="n"/>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Full text</t>
+          <t>Origin of the EWMA baseline and of energy neutral operation, which is what our allocator enforces.</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/WIRELESSVITAE.2009.5172412</t>
+          <t>Abstract only</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/1274858.1274870</t>
         </is>
       </c>
     </row>
@@ -722,49 +759,54 @@
       <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Evaluation and design exploration of solar harvested-energy prediction algorithm</t>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>A. Predicting harvest</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Ali, Al-Hashimi, Recas and Atienza, 2010</t>
+          <t>Prediction and management in energy harvested wireless sensor nodes</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>DATE 2010, pages 142 to 147</t>
+          <t>Recas Piorno, Bergonzini, Atienza and Simunic Rosing, 2009</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Stress tests WCMA at six US measurement sites with a year of data each, at slot lengths from 5 minutes to 1 hour, and measures what a prediction costs on an MSP430.</t>
+          <t>Wireless VITAE 2009</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>MAPE of 3.45 to 8.31 percent at 5 minutes, 6.59 to 17.22 percent at 30 minutes and 8.88 to 21.43 percent at 1 hour, with night excluded. A prediction costs 4 to 9 microjoules, and sampling plus prediction is 2.880 mJ per day, about 0.8 percent of sleep energy.</t>
+          <t>Predicts the next 30 minutes by averaging the same slot over the last 4 days, then scaling that by how today is running against those days. Called WCMA.</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Accuracy depends on the site and on the horizon, and the best parameters differ from one site to another.</t>
+          <t>45 days of one minute data, one panel on a supercapacitor node. Tuned on the same data it was tested on.</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Prediction on the node is effectively free in energy terms. Expect roughly 7 to 21 percent error at the horizons we care about, and retune per node rather than copying published parameters.</t>
+          <t>Average error 9.8 percent, against 28.6 percent for EWMA. On a day the weather turned: 10.20 percent against minus 90.99 percent.</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
+          <t>The cheap baseline our server model has to beat. Read 9.8 percent as optimistic, since it was tuned in sample.</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
           <t>Full text</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/DATE.2010.5457222</t>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/WIRELESSVITAE.2009.5172412</t>
         </is>
       </c>
     </row>
@@ -772,49 +814,54 @@
       <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Online machine learning for 1-day-ahead prediction of indoor photovoltaic energy</t>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>A. Predicting harvest</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Kraemer, Asad, Bach and Renner, 2023</t>
+          <t>Evaluation and design exploration of solar harvested-energy prediction algorithm</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>IEEE Access, volume 11</t>
+          <t>Ali, Al-Hashimi, Recas and Atienza, 2010</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Predicts indoor photovoltaic energy 24 hours ahead at six locations in one building, using 961 days of measurements and online learning with calendar, lag, sun angle and weather forecast inputs. Compares a random forest against persistence and EWMA, and against SVM, XGBoost and neural networks.</t>
+          <t>DATE 2010</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Persistence gave mean total daily errors of 31.52 to 58.54 percent. The random forest improved on persistence by 32 and 23 percent at one window location, 22 and 16 percent at another, and 56 and 47 percent at a hallway lit only by artificial light. EWMA beat persistence at one location only.</t>
+          <t>Takes the WCMA method above and tests how it holds up across different climates, slot lengths and prediction horizons.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Relatively simple machine learning beats a persistence predictor considerably indoors. SVMs, XGBoost and neural networks did not in general score better than the random forest.</t>
+          <t>Six US measurement sites, one year each. Cost measured on an MSP430.</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Indoor only, so it does not transfer directly to our outdoor nodes. It is the clearest case in this set where ML earns its place, and the winner was a tree model rather than a neural network.</t>
+          <t>Error 6.59 to 17.22 percent at 30 minutes and 8.88 to 21.43 percent at 1 hour, depending on site. Costs 4 to 9 microjoules per prediction.</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
+          <t>Sets the accuracy we should expect, and shows prediction on the node is free in energy terms. Retune per site.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
           <t>Full text</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/ACCESS.2023.3267810</t>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/DATE.2010.5457222</t>
         </is>
       </c>
     </row>
@@ -822,49 +869,54 @@
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Statistical and machine learning forecasting methods: concerns and ways forward</t>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>A. Predicting harvest</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Makridakis, Spiliotis and Assimakopoulos, 2018</t>
+          <t>Pro-Energy: a novel energy prediction model for solar and wind energy-harvesting WSNs</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>PLOS ONE, volume 13, issue 3</t>
+          <t>Cammarano, Petrioli and Spenza, 2012</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Compares eight statistical and ten machine learning methods, an LSTM among them, on 1,045 monthly series from the M3 competition, across one step and longer horizons.</t>
+          <t>IEEE MASS 2012</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>One step ahead sMAPE was 7.19 percent for ARIMA, 8.39 percent for a multilayer perceptron and 11.67 percent for the LSTM.</t>
+          <t>Stores whole days of past harvest, then finds the stored day that most resembles today so far and uses the rest of that day as the forecast.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>The machine learning methods were beaten by the statistical ones on both accuracy measures and at every horizon, and the LSTM did not improve accuracy. How well a model fitted the training data did not predict how well it forecast.</t>
+          <t>Solar and wind traces from their own nodes and public stations.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>The direct argument against starting with an LSTM. The caveat is that these are short monthly business series rather than solar data, so it speaks to data hunger more than to solar specifically.</t>
+          <t>Reported as up to 60 percent more accurate than EWMA and WCMA.</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Full text</t>
+          <t>More accurate on paper, but it needs stored day profiles and fails when it matches the wrong day.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1371/journal.pone.0194889</t>
+          <t>Abstract only</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/MASS.2012.6502504</t>
         </is>
       </c>
     </row>
@@ -872,49 +924,54 @@
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>M5 accuracy competition: results, findings, and conclusions</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>A. Predicting harvest</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Makridakis, Spiliotis and Assimakopoulos, 2022</t>
+          <t>A solar altitude angle model for efficient solar energy predictions</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>International Journal of Forecasting, volume 38, issue 4</t>
+          <t>Herreria-Alonso and colleagues, 2020</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Reports the M5 competition: 42,840 hierarchical retail series with price and promotion information, forecast by thousands of entrants.</t>
+          <t>Sensors 20(5)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>All of the top 50 entries beat the best statistical benchmark by more than 14 percent, and the winner by 22.4 percent. Exponential smoothing with the extra variables was 6 percent better than without them, and ARIMAX was 13 percent better than ARIMA.</t>
+          <t>Scales the last measured slot by how much the sun's height changes between now and the target time. Stores no history at all.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>This was the first M competition where all the top performing methods were pure machine learning and beat every statistical benchmark. Most used LightGBM, and learning across many related series helped where individual series were short.</t>
+          <t>NREL Oak Ridge data for 2018, 30 minute slots, horizons of 30 to 120 minutes.</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>This is the setting where ML wins: many related series plus useful external inputs. Five nodes at one site is nothing like 42,840 series, but pooling our nodes and adding weather inputs is the same idea in miniature.</t>
+          <t>Error 10.3 and 5.9 percent lower than a memory heavy Pro-Energy setup at 30 and 60 minutes. Pro-Energy won at 120 minutes.</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
+          <t>Closest published method to the clear sky scaling we plan, and it needs no stored history.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
           <t>Full text</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.ijforecast.2021.11.013</t>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s20051391</t>
         </is>
       </c>
     </row>
@@ -922,49 +979,54 @@
       <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Robustness of predictive energy harvesting systems: analysis and adaptive prediction scaling</t>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>A. Predicting harvest</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Stricker, Da Forno and Thiele, 2022</t>
+          <t>Doctoral thesis on long-term energy-neutral operation of solar harvesting systems</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>IET Computers and Digital Techniques, volume 16, issue 4</t>
+          <t>Buchli, 2015</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Measures how prediction error propagates into scheduler and system performance for solar harvesting nodes, defines a robustness metric, and proposes scaling the forecast down by a factor learned online while holding an energy reserve. Simulated on outdoor and indoor traces, with the model validated on hardware using a 0.95 F supercapacitor.</t>
+          <t>ETH Zurich, thesis 22717</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>An EWMA forecast with only 6 percent mean error still cut weekly usable energy to 66 and 73 percent of what a perfect forecast allowed. EWMA with adaptive scaling reached 3.54 Wh minimum daily energy against 3.14 Wh for the most accurate predictor tested, 13 percent higher. Indoors, persistence had 38 and 56 percent error where EWMA had 54 and 73 percent.</t>
+          <t>Asks whether a more accurate harvest predictor actually produces a better system, by running predictors inside energy management schemes.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>How the scheduler uses a prediction matters more than how accurate the prediction is. A less accurate predictor that is scaled down can beat a more accurate one used at face value.</t>
+          <t>Simulation on multi year solar traces from several locations.</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>The most decision relevant paper in this set. It argues for a simple predictor with a learned safety factor instead of spending our time on a better model.</t>
+          <t>EWMA is only accurate enough over windows of hours. WCMA is about three times more accurate, but that gain does not translate into significant system improvement.</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
+          <t>The warning that chasing predictor accuracy is not the same as improving the node.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
           <t>Full text</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1049/cdt2.12042</t>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.tik.ee.ethz.ch/people/thiele/paper/diss_buchli.pdf</t>
         </is>
       </c>
     </row>
@@ -972,49 +1034,50 @@
       <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Cloudy computing: leveraging weather forecasts in energy harvesting sensor systems</t>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>B. Machine learning</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Sharma, Gummeson, Irwin and Shenoy, 2010</t>
+          <t>A hybrid prediction model based on LSTM, empirical mode decomposition and solar profiles for energy harvesting WSNs</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>IEEE SECON 2010, pages 136 to 144</t>
+          <t>Ge, Nan and Bai, 2019</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Uses National Weather Service sky cover forecasts to predict solar harvest 3 to 72 hours ahead, against a past predicts future baseline, and simulates a sensor network that sets its data rate from the prediction.</t>
+          <t>Energies 12(24)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Between 3 hours and 3 days the forecast based RMSE was under 30 against about 60 for past predicts future. The forecast based system ran out of energy on under 5 percent of days while keeping 80 percent of the baseline data rate, where the history based one ran out on nearly 50 percent of days.</t>
+          <t>Splits the harvest signal into components, then trains an LSTM on them together with profiles of similar past days, predicting an hour ahead.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Beyond a few hours, weather forecasts predict harvest better than a node's own history, and scheduling from them keeps a node alive far more reliably.</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>At the horizons that decide whether a node can run a task later in the day, the gain comes from adding a weather feed, not from a better model.</t>
-        </is>
-      </c>
+          <t>Simulation. Compared against EWMA, WCMA and a plain LSTM.</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n"/>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Full text</t>
+          <t>The one deep learning paper in our domain. It beats statistical predictors only, with no stronger ML baseline tested.</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/SECON.2010.5508260</t>
+          <t>Abstract only</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en12244762</t>
         </is>
       </c>
     </row>
@@ -1022,49 +1085,54 @@
       <c r="A9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Predicting solar generation from weather forecasts using machine learning</t>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>B. Machine learning</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Sharma, Sharma, Irwin and Shenoy, 2011</t>
+          <t>Predicting solar-harvested energy for resource-constrained IoT devices using machine learning</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>IEEE SmartGridComm 2011</t>
+          <t>Khamitov, Orel and Zorbas, 2024</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Predicts solar generation 3 hours ahead at noon from six weather forecast variables plus day of year, comparing linear least squares, support vector regression with and without PCA, a sky cover only model and past predicts future. Trained on January to August 2010 and tested on September and October.</t>
+          <t>IEEE DCOSS-IoT 2024</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Test RMSE in W per square metre: 128 for SVR with PCA, 130 for linear least squares, 163 for SVR with an RBF kernel, 175 for the sky cover model and 261 for past predicts future.</t>
+          <t>Predicts harvested energy from time of day and the device's own light readings, with no weather input, comparing quantile regression, random forest, gradient boosting and a small neural network.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Machine learning on several weather variables predicts generation considerably better than a sky cover model or the node's own history.</t>
+          <t>Includes an ESP32 prototype running the models.</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>The algorithm barely mattered here. SVR with PCA beat plain linear regression by 2 W per square metre, so the variables did the work, not the model.</t>
+          <t>Random forest and gradient boosting were best: 21.49 percent sMAPE at 30 minutes, rising to 32.53 and 36.33 percent at 5 hours.</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Full text</t>
+          <t>Same problem as ours, on a microcontroller. Tree models won, and error roughly doubles from 30 minutes to 5 hours.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/SmartGridComm.2011.6102379</t>
+          <t>Abstract only</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/DCOSS-IoT61029.2024.00103</t>
         </is>
       </c>
     </row>
@@ -1072,49 +1140,54 @@
       <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>An energy-aware task scheduler for energy-harvesting batteryless IoT devices</t>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>B. Machine learning</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Sabovic, Sultania, Delgado, De Roeck and Famaey, 2022</t>
+          <t>Online machine learning for 1-day-ahead prediction of indoor photovoltaic energy</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>IEEE Internet of Things Journal, volume 9, issue 22</t>
+          <t>Kraemer, Asad, Bach and Renner, 2023</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>A task scheduler for batteryless devices. Each task gets a required start voltage from a capacitor model, and the device sleeps and re-measures until it can finish the task before its deadline. Tested on real hardware with an e-peas harvester and an amorphous silicon panel under controlled light, with capacitors from 4.7 to 20 mF.</t>
+          <t>IEEE Access 11</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>The scheduled device stayed awake for the entire experiment and avoided power failures completely, and executed more cycles than the energy unaware scheduler at 10 mF or less with 40 microamps of harvest. The measurement divider drew about 1.5 mA while sampling.</t>
+          <t>Predicts tomorrow's 24 hourly harvest values for indoor panels, training online as data arrives, using calendar, past values, sun angle and weather forecasts.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Checking measured storage voltage against a per task threshold is enough to avoid power failures. The authors state that they did not consider a predictive approach.</t>
+          <t>961 days of measurements at six locations in one building.</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>The closest hardware match to our nodes, and it supports the energy gate we designed. The divider current is a direct warning for our own voltage sensing bodge.</t>
+          <t>Random forest beat the same hour yesterday by 22 to 32 percent near windows and by 56 percent in a hallway with artificial light only. SVM, XGBoost and neural networks did not beat the random forest.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
+          <t>Indoors only, so not a direct match, but the clearest case where ML earns its place, and a tree model won.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
           <t>Full text</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/JIOT.2022.3185321</t>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ACCESS.2023.3267810</t>
         </is>
       </c>
     </row>
@@ -1122,49 +1195,54 @@
       <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Energy-aware packet schedulers for battery-less LoRaWAN nodes</t>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>B. Machine learning</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Capuzzo, Delgado, Famaey and Zanella, 2022</t>
+          <t>Uncertainty-aware energy harvest prediction and management for IoT devices</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>arXiv preprint 2212.09453</t>
+          <t>Yamin and Bhat, 2023</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Compares seven packet scheduling policies for a batteryless LoRaWAN node that differ only in how they estimate harvest: an oracle with true future harvest, a fixed voltage threshold, an assumption of zero harvest, short moving averages, and an energy unaware baseline. Simulated in ns-3 on four real indoor solar traces.</t>
+          <t>ACM TODAES</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>The energy unaware scheduler sent 20 to 40 percent fewer packets than the oracle, and the fixed threshold about 10 percent fewer. Assuming zero harvest and averaging the last 5 seconds were both almost optimal. With a 2 mF capacitor the zero harvest policy sent nothing at all, because its threshold could never be reached.</t>
+          <t>Predicts both the expected harvest and how uncertain that prediction is, then feeds both into an optimiser that decides how much energy to spend.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Energy aware scheduling raises how many packets a batteryless LoRaWAN node can send, and simple harvest estimates come close to an oracle that knows the future.</t>
+          <t>Five years of solar data. Low power neural network intended to run on the device.</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Direct LoRaWAN precedent. Our gate does not need a sophisticated forecast, but a rule that is too conservative can block the work entirely.</t>
+          <t>Mean error 3.4 J at 80 percent coverage, and energy allocations within 2.5 J of what an oracle would have chosen.</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Preprint, full text</t>
+          <t>The shape we want: predict a range rather than a number, and let the allocator plan against the low end.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2212.09453</t>
+          <t>Abstract only</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3606372</t>
         </is>
       </c>
     </row>
@@ -1172,49 +1250,54 @@
       <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>ACES: automatic configuration of energy harvesting sensors with reinforcement learning</t>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>B. Machine learning</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Fraternali, Balaji, Agarwal and Gupta, 2020</t>
+          <t>Cloudy computing: leveraging weather forecasts in energy harvesting sensor systems</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>ACM Transactions on Sensor Networks, volume 16, issue 4</t>
+          <t>Sharma, Gummeson, Irwin and Shenoy, 2010</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Uses tabular Q learning on a server to set the sensing period of indoor light powered supercapacitor nodes. The state is light level, supercapacitor voltage and a weekday flag, and training uses a simulator built from datasheets plus 15 days of each node's own light data. Deployed on 60 nodes for two weeks.</t>
+          <t>IEEE SECON 2010</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Nodes stopped operating 0.1 percent of the time in the deployment. In simulation the mean sampling period was 71 s against 107 s for the authors' own rule based manager and 100 to 112 s for three earlier RL methods. Learning day by day ran two nodes flat in the first days until transfer learning was added, and a four day server outage killed three nodes.</t>
+          <t>Predicts harvest by taking a clear day profile and shading it by the cloud cover in a public weather forecast, instead of using the node's own history.</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Reinforcement learning can configure harvesting sensors better than hand written rules, as long as it is trained on a simulator first and protected while it learns.</t>
+          <t>One rooftop panel, 3 to 72 hour horizons, plus a simulated sensor network that sets its data rate from the prediction.</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Shows RL is possible on hardware like ours, and what it costs: a simulator, per node data, and a way to survive exploration. Not a first step for a project our size.</t>
+          <t>Forecast error about half that of history based prediction between 3 hours and 3 days. Nodes ran out of energy on under 5 percent of days, against nearly 50 percent with history based prediction.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
+          <t>Beyond a couple of hours, the win comes from adding a weather feed, not from a better model.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
           <t>Full text</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1145/3404191</t>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/SECON.2010.5508260</t>
         </is>
       </c>
     </row>
@@ -1222,45 +1305,54 @@
       <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>History and trends in solar irradiance and PV power forecasting: a preliminary assessment and review using text mining</t>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>B. Machine learning</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Yang, Kleissl, Gueymard, Pedro and Coimbra, 2018</t>
+          <t>Predicting solar generation from weather forecasts using machine learning</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Solar Energy, volume 168, pages 60 to 101</t>
+          <t>Sharma, Sharma, Irwin and Shenoy, 2011</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>A text mining review of the solar irradiance and PV forecasting literature, covering how methods are grouped, how they are evaluated, and what the field treats as standard practice.</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n"/>
+          <t>IEEE SmartGridComm 2011</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Trains regression models on six weather forecast variables plus day of year to predict generation 3 hours ahead.</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Quoting the review: the proper implementation of any of these methods yields similar forecasting skills, as long as overfitting is prevented. It also notes that in their simplest forms, ML methods are statistical methods, and that almost every statistical and machine learning solar forecasting paper removes the diurnal cycle.</t>
+          <t>Trained on January to August 2010, tested on September and October.</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>This answers the stochastic versus ML question directly. The split is not a real one, and normalising out the clear sky curve matters more than the family of model we choose.</t>
+          <t>Error in W per square metre: 128 for SVR with PCA, 130 for plain linear regression, 175 for a cloud cover only model, 261 for using history.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
+          <t>The model barely mattered. SVR beat linear regression by 2 units, while the weather variables cut error by half.</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
           <t>Full text</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.solener.2017.11.023</t>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/SmartGridComm.2011.6102379</t>
         </is>
       </c>
     </row>
@@ -1268,49 +1360,54 @@
       <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>A meta-analysis of solar forecasting based on skill score</t>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Nguyen and Musgens, 2022</t>
+          <t>Robustness of predictive energy harvesting systems: analysis and adaptive prediction scaling</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>arXiv preprint 2208.10536</t>
+          <t>Stricker, Da Forno and Thiele, 2022</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>A meta analysis of deterministic solar forecasting. The authors screened 1,447 papers, read 320 in full, and analysed 4,687 reported results for what drives forecast skill.</t>
+          <t>IET Computers and Digital Techniques 16(4)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>4,687 data points from 320 papers. Overfitting appeared once training sets ran longer than about 2,000 days.</t>
+          <t>Measures how much system performance is lost as forecast error grows, then deliberately scales the forecast down by a factor learned online and keeps an energy reserve.</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Forecast horizon has a central impact and dominates the other factors. Ensemble and hybrid models were the most accurate at every horizon, sky and satellite images were the most useful inputs intra day, and numerical weather predictions with local measurements were the most useful day ahead.</t>
+          <t>Outdoor and indoor traces, with the model validated on hardware using a 0.95 F supercapacitor.</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Tells us to choose the method for our horizon rather than in general, and that adding inputs beats adding model complexity.</t>
+          <t>A forecast with only 6 percent mean error still cost about a third of weekly usable energy. A scaled down EWMA beat the most accurate predictor tested by 13 percent.</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Preprint, full text</t>
+          <t>The most useful paper here. It says spend the effort on the safety margin, not on the predictor.</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2208.10536</t>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1049/cdt2.12042</t>
         </is>
       </c>
     </row>
@@ -1318,54 +1415,605 @@
       <c r="A15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>An energy-aware task scheduler for energy-harvesting batteryless IoT devices</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Sabovic, Sultania, Delgado, De Roeck and Famaey, 2022</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>IEEE IoT Journal 9(22)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Gives every task a start voltage it must see before running, computed from a capacitor model, and makes the device wait and re-measure until it can finish the task.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Real hardware: nRF52840, e-peas harvester, amorphous silicon panel, capacitors of 4.7 to 20 mF.</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>No power failures at all across the experiment, and more completed cycles than an energy unaware scheduler. Their measurement divider drew about 1.5 mA while sampling.</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Closest hardware match to our node, and it works with no prediction at all. The divider current is a warning for our voltage sensing bodge.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/JIOT.2022.3185321</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Energy-aware packet schedulers for battery-less LoRaWAN nodes</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Capuzzo, Delgado, Famaey and Zanella, 2022</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2212.09453</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Compares seven ways of deciding whether a LoRaWAN node can afford to transmit, from an oracle that knows future harvest down to a fixed voltage threshold.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>ns-3 simulation on four real indoor solar traces, one node.</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Ignoring energy cost 20 to 40 percent of packets against the oracle. Assuming zero harvest, or averaging the last 5 seconds, came out almost as good as the oracle.</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Direct LoRaWAN precedent. A simple estimate is enough, but an overly cautious rule can block all work.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Preprint, full text</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2212.09453</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Optimal energy-aware task scheduling for batteryless IoT devices</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Delgado and Famaey, 2021</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>IEEE TETC</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Solves task scheduling exactly, as a mathematical optimisation that maximises completed work while keeping capacitor voltage inside its limits.</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Simulation with an nRF52840 profile, 4.7 mF, harvest of 0.1 to 5 mW.</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Completed 36 of 41 tasks against 21 for a scheduler that ignores energy. Zero power failures, but only when future harvest is known perfectly. A look ahead of 8 tasks was enough.</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Use it as the upper bound when we score our rule, not as something to deploy.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/TETC.2021.3086144</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Energy-aware adaptive scheduling for battery-less 6TiSCH routers</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Van Leemput, Famaey, Hoebeke and De Poorter, 2024</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>IEEE Access 12</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>A central manager collects voltage and harvest telemetry from each node, predicts each node's capacitor voltage 15 minutes ahead, and throttles the ones that would run flat.</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Cooja simulation, 200 mF storage, harvest of 200 to 1200 microwatts.</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Reporting success and uptime both improved by 12 percent, reaching about 90 percent. The algorithm itself cost 87.94 nW, and latency rose 32.28 percent.</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>The closest published design to ours: a server predicting each node's voltage and scheduling from it. Simulation only, and 6TiSCH rather than LoRaWAN.</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ACCESS.2024.3508540</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Energy-aware task allocation for energy harvesting sensor networks</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Edalat and Motani, 2016</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>EURASIP JWCN 2016</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Allocates tasks across several harvesting nodes from a central point, scoring each node by task length divided by the energy it has available.</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Simulation. Forecasts come from a combined autoregressive and WCMA predictor.</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>A simple greedy version of the rule reached up to 70 percent of what exact optimisation achieved, and a genetic algorithm reached 82 percent.</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>The only paper here that allocates tasks across several nodes, which is our exact problem. Our scoring rule comes from it.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s13638-015-0490-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Managing task execution for unknown workloads in batteryless IoT</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Nasser, Moura, Singh, Weyn and Famaey, 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2606.24340</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Compares ways of deciding whether to run or skip a task when the task's energy cost is not known in advance, including reinforcement learning and fixed thresholds.</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Simulation driven by real solar data and LoRa transmission profiles, capacitors of 0.5 to 10 F.</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Their lightweight prediction method came close to oracle throughput, and devices with larger energy buffers did fine on simple static thresholds.</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Recent and close to our setup. With a big enough capacitor, a static threshold is enough.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Preprint, abstract only</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2606.24340</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>ACES: automatic configuration of energy harvesting sensors with reinforcement learning</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Fraternali, Balaji, Agarwal and Gupta, 2020</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>ACM TOSN 16(4)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Learns, by trial and error on a server, how often each node should sample, from its light level, capacitor voltage and whether it is a weekday.</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Simulator built from datasheets plus 15 days of each node's light data, then 60 nodes deployed for two weeks.</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Nodes were dead 0.1 percent of the time, and sampled more often than the authors' own rule based manager. While learning day by day, two nodes ran flat, and a four day server outage killed three more.</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Shows RL works on hardware like ours, and what it costs: a simulator, per node data, and protection while it explores.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3404191</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>C. Using the prediction</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Adaptive power management in solar energy harvesting sensor node using reinforcement learning</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Shresthamali, Kondo and Nakamura, 2017</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>ACM TECS 16(5s)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Learns a duty cycle policy from battery level, harvested energy and the day's weather forecast, trained offline before deployment.</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Simulation on Tokyo solar data for training, tested on a different year and a different city.</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Deviation from energy neutrality over 30 days: 5.27 percent for the learned policy, 23.82 percent for a naive rule, 3.46 percent for a planner given the true future. On single days and at an unseen site it matched that planner.</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>RL ties a planner that knows the future, but its large margin is only over a naive rule, not over a good one.</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3126495</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>D. Our site and ground rules</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Impact of dust on the performance of solar photovoltaic (PV) systems under United Arab Emirates weather conditions</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Hachicha, Al-Sawafta and Said, 2019</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Renewable Energy, volume 141, pages 287 to 297</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Indoor and outdoor experiments in Sharjah characterising deposited dust, with particle sizes from 1.61 to 38.40 micrometres, and its effect on PV electrical performance. Includes five months of outdoor exposure and a comparison of panel tilt angles.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Normalised power fell 1.7 percent per g per square metre of dust. Efficiency loss by tilt was 37.63 percent for horizontal panels, 14.11 percent at 25 degrees and 10.95 percent at 45 degrees. Over five months outdoors, soiling losses rose 12.7 percent as dust density reached 5.44 g per square metre.</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Dust is a large and tilt dependent loss under UAE conditions, and a linear model of dust density predicts the drop in performance.</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Our panels are glued flat to the lid, which is the worst case in this study. It also gives a model something real to learn: a per node soiling factor that decays between cleanings.</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Renewable Energy 141</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Measures how much power dust costs a PV panel in Sharjah, and how much of that depends on the angle the panel is mounted at.</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Indoor and outdoor experiments in Sharjah, including five months of outdoor exposure.</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Power fell 1.7 percent per gram of dust per square metre. Loss by tilt: 37.63 percent horizontal, 14.11 percent at 25 degrees, 10.95 percent at 45 degrees. Soiling losses rose 12.7 percent over five months.</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Our panels sit flat on the lid, which is the worst case measured here. It also gives a model something real to learn between cleanings.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>Abstract only</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.renene.2019.04.004</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>D. Our site and ground rules</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>History and trends in solar irradiance and PV power forecasting</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Yang, Kleissl, Gueymard, Pedro and Coimbra, 2018</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Solar Energy 168</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Reviews how the solar forecasting field works: how methods are grouped, how they are evaluated, and what counts as standard practice.</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Text mining review of the published literature.</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Says any of these methods, properly implemented, gives similar skill, and that simple ML methods are statistical methods. It settles the stochastic versus ML question.</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.solener.2017.11.023</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>D. Our site and ground rules</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>A meta-analysis of solar forecasting based on skill score</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Nguyen and Musgens, 2022</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2208.10536</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Collects the results reported across the solar forecasting literature and analyses what actually drives forecast accuracy.</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>1,447 papers screened, 320 read in full, 4,687 reported results analysed.</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Forecast horizon dominates every other factor. Combined and hybrid models were most accurate at every horizon. Training sets longer than about 2,000 days started to overfit.</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Choose the method for our horizon rather than in general, and expect more from better inputs than from a bigger model.</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Preprint, full text</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2208.10536</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J15"/>
+  <autoFilter ref="A1:K25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1376,238 +2024,115 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="74" customWidth="1" min="2" max="2"/>
-    <col width="74" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>What we found</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>What it rests on</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>How sure we are</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>No study we read shows an LSTM beating simpler models at the horizons a task allocator needs. Where deep learning did appear at node level, it was only compared against EWMA or WCMA.</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Makridakis 2018 (LSTM sMAPE 11.67 against ARIMA 7.19). We found no node level study comparing an LSTM against gradient boosting or a weather driven regression.</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Well supported, with the caveat that M3 is monthly business data, not solar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Where machine learning does win, the winner is usually a tree model, and the gain comes from the inputs rather than the algorithm.</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Kraemer 2023 (random forest beat SVM, XGBoost and neural networks indoors), Sharma 2011 (SVR beat linear regression by 2 W per square metre while both beat history by a wide margin), M5 2022 (LightGBM plus covariates).</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Well supported across three papers.</t>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cross-domain evidence: does machine learning beat statistical forecasting in general?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>These two are not energy harvesting papers. They are business and retail forecasting competitions, and they are the standard citation for whether machine learning beats statistical methods when data is short or plentiful. They are kept off the Papers sheet for that reason. Drop this sheet if it distracts from the domain review.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>How the scheduler uses a forecast matters more than how accurate the forecast is.</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Stricker 2022 (6 percent mean error still cost about a third of usable energy; a scaled down EWMA beat the most accurate predictor by 13 percent), Capuzzo 2022 (zero harvest and 5 second average both almost optimal against an oracle).</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Well supported, and it is the finding that shapes our design.</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Authors, year</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>What it tested</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>What we take from it</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>4</v>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Statistical and machine learning forecasting methods: concerns and ways forward</t>
+        </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Simple threshold rules on measured storage voltage avoid power failures on hardware very like ours, without any prediction at all.</t>
+          <t>Makridakis, Spiliotis and Assimakopoulos, 2018</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Sabovic 2022 (real e-peas hardware, no power failures, and the authors state they did not consider a predictive approach).</t>
+          <t>Eight statistical methods against ten machine learning ones, an LSTM among them, on 1,045 monthly business series.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Demonstrated on hardware.</t>
+          <t>One step error was 7.19 percent for ARIMA, 8.39 percent for a neural network and 11.67 percent for the LSTM. The ML methods lost at every horizon.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>With short series, an LSTM is a poor first choice. Business data, not solar, so treat it as a statement about data hunger.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>5</v>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>M5 accuracy competition: results, findings and conclusions</t>
+        </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Forecasts earn their place at horizons beyond a couple of hours, and that is where weather data, not model complexity, does the work.</t>
+          <t>Makridakis, Spiliotis and Assimakopoulos, 2022</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Sharma 2010 (battery depleted on under 5 percent of days with forecasts against nearly 50 percent without), Nguyen and Musgens 2022 (horizon dominates all other factors).</t>
+          <t>42,840 related retail sales series with price and promotion data, forecast by thousands of entrants.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Well supported.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Reinforcement learning is a research project in its own right, and it drains supercapacitors while it learns.</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Fraternali 2020 (two nodes ran flat during day by day learning; a server outage killed three more; needed a simulator plus 15 days of per node data).</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Clear enough that we are not attempting it now.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Our hardware, not the model, is the binding limit. One ENS160 reading needs about 21 J out of storage, and the 0.22 F supercapacitor holds about 0.56 J between the PMIC thresholds as rev 1 is wired.</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Our own calculation from the ENS160 datasheet (29 mA for a 3 minute warm up at 3.3 V) and the stored energy formula. Not from any paper.</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Calculation only. PPK2 measurements will replace it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>The ENS160 has no cheap measuring mode, so the cost per reading cannot be tuned away in firmware.</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>ScioSense ENS160 datasheet version 1.3: average current 0.01 mA in deep sleep, 2 mA typical in idle, 29 mA in standard mode, with a 79 mA peak for under 5 ms. Warm up is required after idle periods as well as after power off.</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>From the datasheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Each ENS160 needs a one time 24 hour burn in on a bench supply, or every duty cycled field reading comes back at start up quality.</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>ScioSense ENS160 datasheet version 1.3: status is stored in non volatile memory only after 24 hours of continuous operation, and if unpowered before that the sensor resumes initial start up mode.</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>From the datasheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Dust is the local variable worth modelling in Sharjah, and our flat panel mounting is the worst case for it.</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Hachicha 2019 (1.7 percent loss per g per square metre; 37.63 percent loss horizontal against 10.95 percent at 45 degrees), plus our enclosure design, which glues the panels flat to the lid.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Paper read at abstract level; the mounting is our own design choice.</t>
+          <t>Every top entry was pure machine learning and beat all statistical benchmarks, the winner by 22.4 percent. Most used gradient boosting.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>ML wins when you have many related series and useful extra inputs. Five nodes at one site is nowhere near that, but pooling nodes and adding weather is the same idea.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1618,7 +2143,269 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>What we found</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Which papers say so</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>How sure we are</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>No paper in our domain shows deep learning beating simpler methods. The one LSTM study here only compared itself against EWMA and WCMA.</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Ge 2019 (row 7). Cross domain: Makridakis 2018 on the Background sheet.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Supported, though the domain evidence is thin in both directions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Where machine learning does win on harvesting data, tree models win, not neural networks.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Khamitov 2024 (row 8), Kraemer 2023 (row 9).</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Two papers, both clear on this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Inputs beat algorithms. Adding a weather feed halved error where a fancier model changed almost nothing.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Sharma 2010 (row 11), Sharma 2011 (row 12), Nguyen and Musgens 2022 (row 24).</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Well supported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>How the scheduler uses the forecast matters more than the forecast's accuracy.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Stricker 2022 (row 13), Capuzzo 2022 (row 15), Buchli 2015 (row 6).</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Well supported, and it shapes our design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>A voltage threshold with a margin, and no prediction at all, already avoids power failures on hardware like ours.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Sabovic 2022 (row 14), Nasser 2026 (row 19).</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Demonstrated on hardware in row 14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Reinforcement learning matches a planner that knows the future, but drains supercapacitors while it learns.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Fraternali 2020 (row 20), Shresthamali 2017 (row 21).</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Clear enough that we are not attempting it now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Error grows fast with horizon, so predict over minutes to a couple of hours, not days.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Ali 2010 (row 3), Khamitov 2024 (row 8), Nguyen and Musgens 2022 (row 24).</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Consistent across three papers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Our hardware is the binding limit, not the model. One ENS160 reading needs about 21 J from storage, and the 0.22 F supercapacitor holds about 0.56 J between the PMIC thresholds as rev 1 is wired.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Ours, calculated from the ENS160 datasheet and the stored energy formula. Not from any paper.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Calculation only. PPK2 measurements will replace it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>The ENS160 has no cheap measuring mode, so the cost per reading cannot be tuned away in firmware.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>ScioSense ENS160 datasheet v1.3: 0.01 mA deep sleep, 2 mA idle, 29 mA standard, 79 mA peak under 5 ms. Warm up is needed after idle as well as after power off.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>From the datasheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Each ENS160 needs one 24 hour burn in on a bench supply, or every duty cycled reading comes back at start up quality.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>ScioSense ENS160 datasheet v1.3: status is stored in non volatile memory only after 24 hours of continuous operation.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>From the datasheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Dust is the local variable worth modelling here, and our flat panel mounting is the worst case for it.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Hachicha 2019 (row 22), plus our own enclosure design.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Paper read at abstract level. The mounting is our choice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1645,7 +2432,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Do we continue with a stochastic or statistical approach, or move to machine learning?</t>
+          <t>Do we continue with a statistical approach, or move to machine learning?</t>
         </is>
       </c>
     </row>
@@ -1657,110 +2444,348 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Statistical baseline plus a rule based allocator first. Keep one machine learning model as a challenger, judged on the same test as the baseline. Do not start with an LSTM.</t>
+          <t>Statistical baseline plus a rule based allocator first. One machine learning model as a challenger, judged on the same test. No LSTM, no reinforcement learning.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Why, in one line</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>At our horizons and our data volume, the papers show simple methods are hard to beat, and the scheduler's safety margin matters more than forecast accuracy.</t>
+          <t>At our horizon and our data volume, the domain papers show simple methods are hard to beat, and the safety margin matters more than the forecast.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>What the baseline is</t>
+          <t>The baseline</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>A clear sky curve for Sharjah, scaled by the clear sky index measured over recent slots, plus persistence for the next slot, and a per node factor learned from predicted against achieved harvest. That factor absorbs soiling, shading and ageing.</t>
+          <t>A clear sky curve for Sharjah, scaled by the clear sky index measured over recent slots, plus a per node factor learned from predicted against achieved harvest. That factor absorbs soiling, shading and ageing.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>What the allocator does</t>
+          <t>The allocator</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Two gates. The cheap SHT41 reading is an energy question: run it if stored energy minus the task leaves a reserve. The ENS160 reading is a power question until we fit a larger capacitor: run it only if predicted harvest power holds above the load for the warm up, using a low quantile rather than an average.</t>
+          <t>Two gates. The SHT41 reading is an energy question: run it if stored energy leaves a reserve. The ENS160 reading is a power question until a larger capacitor is fitted: run it only if predicted harvest power holds through the warm up, judged on a low quantile rather than an average.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>The one ML model worth trying</t>
+          <t>The ML challenger</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>A quantile gradient boosting model shared across all five nodes, with clear sky, dust and aerosol inputs from the free Open-Meteo air quality feed. Scored on how many ENS160 runs complete rather than on RMSE.</t>
+          <t>A quantile gradient boosting model shared across all five nodes, with clear sky, dust and aerosol inputs from the free Open-Meteo air quality feed. Scored on completed ENS160 runs, not on RMSE.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>What we are not doing</t>
+          <t>What would change our minds</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>LSTM or other deep learning as the main predictor, and reinforcement learning. Neither is required for the project, and neither is supported by what we read for a fleet this size.</t>
+          <t>If the rule is tuned and ENS160 runs still abort often, or if error tracks dust loading more than anything else, the gradient boosting model becomes worth building.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>What would change our minds</t>
+          <t>How we judge it</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>If the rule is tuned and ENS160 runs still abort often, or if error tracks dust loading more than anything else, then the gradient boosting model with dust inputs becomes worth the effort.</t>
+          <t>Completed against aborted ENS160 runs, brown outs and missed uplinks, on the same replayed data for every method. Forecast error in joules or watts as a secondary measure, never MAPE, which breaks down at night.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>How we will judge it</t>
+          <t>For the report</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Completed against aborted ENS160 runs, brown outs, and missed uplinks, on the same replayed data for every method. Forecast error in joules or watts as a secondary measure, never MAPE, which breaks down at night.</t>
+          <t>Comparing a statistical baseline against an ML challenger on our own data is a result either way. If the baseline wins, that is a finding, and rows 6, 13 and 15 predict it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Why it appears here</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>The no change forecast. Either the next slot equals the last measured slot, or today's 09:00 equals yesterday's 09:00.</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>The floor every method is measured against. Free, and harder to beat than people expect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>EWMA</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Exponentially weighted moving average. Keeps one running average per time of day, updated each day with a decay factor, so it reflects many past days.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>The original predictor for harvesting nodes, from row 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>WCMA</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Weather conditioned moving average. The EWMA style profile, scaled by how today's recent slots compare with the same slots on past days.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Rows 2 and 3. The standard statistical baseline in this field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Pro-Energy</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Stores whole past days and predicts using the stored day that best matches today so far.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Row 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Clear sky index</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Measured output divided by what a clear sky would give at that moment. Strips out the sun's daily arc so only the weather is left.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>The basis of our planned baseline, and standard practice per row 23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Skill score</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>How much better a forecast is than a reference, usually persistence. Zero means no better than doing nothing.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>How rows 23 and 24 compare methods across studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>MAPE and sMAPE</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Average percentage error. Both break down when the true value is near zero, which is every night for solar.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Why we will report errors in joules or watts instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Quantile forecast</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>A forecast that gives a range, for example the value harvest will exceed 90 percent of the time, instead of a single number.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>What the allocator should use, per row 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>A method given the true future, used as an upper bound. Not something you can deploy.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Rows 15, 16 and 21 measure against one.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Honest framing for the report</t>
+          <t>Energy neutral operation</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Comparing a statistical baseline against a machine learning challenger on our own data is a result either way. If the baseline wins, that is a finding, and the papers here predict it.</t>
+          <t>Spending on average no more energy than the node harvests, so it runs indefinitely.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>The goal set out in row 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Batteryless</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>A node storing energy only in a capacitor, so it loses power regularly and must survive that.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Rows 14 to 19, and our own node.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Every claim on this sheet traces to the Papers or What we found sheets, except the design choices, which are ours.</t>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Duty cycle</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>The fraction of time a node is awake or sensing. The usual thing these papers control.</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Most of group C tunes this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Reinforcement learning</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Learning a policy by trying actions and receiving rewards, rather than predicting a value.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Rows 20 and 21.</t>
         </is>
       </c>
     </row>

</xml_diff>